<commit_message>
Anthropic v0.1.3 A 步驟 7：報告、對照 Excel、CHANGELOG、進度檔
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012m1PVCRgcynaQmdau6562e
</commit_message>
<xml_diff>
--- a/anthropic/docs/reports/20261022_v0.1.3-A_對照.xlsx
+++ b/anthropic/docs/reports/20261022_v0.1.3-A_對照.xlsx
@@ -519,7 +519,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>對照（U2）：Lambda 揭露 MW ÷ 1000 vs 模型 Lambda 供給 GW（金額回推；D 欄＝揭露，E–I＝模型）</t>
+          <t>供給 GW（U2 新法）：Nscale Monarch＝揭露 MW ÷ 1000 × IT 換算 × 爬坡 × 期間</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -527,27 +527,27 @@
           <t>GW</t>
         </is>
       </c>
-      <c r="E2" s="3" t="n">
-        <v>0.35</v>
+      <c r="E2" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="3" t="n">
-        <v>0.175</v>
+      <c r="G2" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>0.35</v>
+        <v>0.23</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>0.35</v>
+        <v>0.46</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>0.35</v>
+        <v>0.46</v>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>D10：GW 由金額回推並與既有揭露 GW 對照（不校準）</t>
+          <t>揭露容量（SRC_ANT 的 MW，Verified／Interested-party）；期間＝Inputs 起始年至結束年（U2）；u2_method＝1 時進入供給</t>
         </is>
       </c>
     </row>
@@ -564,25 +564,35 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>對照（U2）：Lambda 模型峰值 GW ÷ 揭露 GW</t>
+          <t>供給 GW（U2 新法）：Lambda＝揭露 MW ÷ 1000 × IT 換算 × 爬坡 × 期間</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>倍</t>
+          <t>GW</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
-      <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0.35</v>
+      </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>&gt; 1＝金額回推的 GW 大於揭露（合約價 12 偏低或『最高 86』含未計容量）</t>
+          <t>揭露容量（SRC_ANT 的 MW，Verified／Interested-party）；期間＝Inputs 起始年至結束年（U2）；u2_method＝1 時進入供給</t>
         </is>
       </c>
     </row>
@@ -9622,7 +9632,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>計入則第 1 層缺口縮小約 20.3</t>
+          <t>計入則第 1 層起算現金多 20.28，累計外部資金需求最多減少同額</t>
         </is>
       </c>
     </row>

</xml_diff>